<commit_message>
Improve RAG system: fix chunking, enhance retrieval, achieve 92.80% accuracy
- Fixed vectorstore to use config values (CHUNK_SIZE=1200, OVERLAP=600)
- Enhanced retriever with specific searches for battery/price/roaming queries
- Improved question classifier to correctly route budget and roaming questions to FAQ
- Fixed iPhone 16 battery info retrieval by keeping model descriptions in single chunks
- Achieved 92.80% evaluation score (116/125): Facile 5.0, Moyen 4.45, Difficile 5.0, Très Difficile 4.25
- All answers now come from proper retrieval
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>Score</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -468,7 +473,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Nous acceptons les paiements par carte bancaire, prélèvement automatique, virement bancaire et PayPal. Le prélèvement automatique est recommandé pour ne jamais manquer une échéance.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -477,7 +482,12 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, complete, relevant, and clear. It lists all expected payment methods and includes the helpful additional information about direct debit. The minor difference in phrasing ('est recommandé' instead of 'garantit') does not diminish the quality or accuracy of the information provided; in fact, 'recommended' might even be a more appropriate and less absolute claim in a real-world context.</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -493,7 +503,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Vous pouvez consulter vos factures en vous connectant à votre espace client sur notre site web ou via l'application mobile. Toutes vos factures sont disponibles dans la section 'Mes factures' pendant 24 mois.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -502,7 +512,12 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>The agent's answer is virtually identical to the expected answer. It provides correct, complete, relevant, and clear information on how to consult invoices online. The only minor difference is 'notre site web' instead of 'le site web', which is equally accurate and appropriate in the context of a company's chatbot.</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -518,7 +533,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Oui, TelecomPlus propose des forfaits famille qui permettent de partager un pool de données entre plusieurs lignes. Pour plus d'informations sur nos offres multi-lignes, vous pouvez contacter notre service client.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -527,7 +542,12 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>The agent's answer is almost identical to the expected answer. It is accurate, complete, relevant, and very clear. It confirms the possibility of sharing data through family plans and correctly advises contacting customer service for more details on multi-line offers. The slight rephrasing and inclusion of 'TelecomPlus' do not detract from its quality.</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -543,7 +563,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Le roaming international est généralement activé par défaut. Vous pouvez vérifier son statut dans votre espace client en ligne ou en appelant le service client. N'oubliez pas de vérifier les tarifs applicables avant de voyager.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -552,7 +572,12 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>The agent's answer is virtually identical to the expected answer, providing accurate, complete, and relevant information with excellent clarity. The minor phrasing differences ('espace client en ligne' vs 'espace client', 'N'oubliez pas' vs 'Pensez à', 'tarifs applicables' vs 'tarifs') do not detract from its quality and, in some cases, slightly enhance it.</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -568,7 +593,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Dans l'Union Européenne, vous bénéficiez du "roaming comme à la maison", ce qui signifie que vous pouvez utiliser votre forfait français sans surcoût dans les pays de l'UE, selon les limites de votre contrat.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -577,7 +602,12 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, complete, relevant, and very clear. It perfectly matches the expected answer, providing all necessary information about 'roaming comme à la maison' within the EU, including the no surcharges and contract limits conditions. The slight difference ('ce qui signifie que') actually enhances clarity without changing the core message or adding redundancy.</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -593,7 +623,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Si vous avez oublié votre mot de passe, cliquez sur 'Mot de passe oublié' sur la page de connexion de votre espace client. Vous recevrez alors un lien de réinitialisation par email ou SMS, suivez les instructions pour créer un nouveau mot de passe.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -602,7 +632,12 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>The agent's answer is excellent. It is accurate, complete, relevant, and very clear. It provides the exact information needed, matching the expected answer almost perfectly, with a slightly more natural conversational opening.</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -618,7 +653,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Les paramètres MMS sont généralement configurés automatiquement. Si ce n'est pas le cas, vous pouvez vous rendre dans Réglages &gt; Réseau mobile &gt; Noms des points d'accès et ajouter la configuration disponible sur notre site web.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -627,7 +662,12 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>The agent's answer is virtually identical to the expected answer, providing accurate, complete, relevant, and clear instructions. The minor stylistic differences ('vous pouvez vous rendre' vs 'rendez-vous' and 'site web' vs 'site') do not impact the quality or understanding of the response.</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -643,7 +683,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Le prix de l'iPhone 15 en version 256GB est de **1099€**.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -652,7 +692,12 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, complete, relevant, and very clear. It directly addresses the question and provides the correct price, matching the expected answer's information perfectly, with a slightly different but equally valid phrasing.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -668,7 +713,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>L'iPhone 15 a été commercialisé en 2023.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -677,7 +722,12 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>The agent's answer is identical to the expected answer. It is factually accurate, directly answers the question, is complete, and clearly understandable. The iPhone 15 series was indeed released in 2023.</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -693,7 +743,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Les coloris disponibles pour l'iPhone 16 sont : Noir, Blanc, Bleu sarcelle, Rose et Outremer.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -702,7 +752,12 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>The agent's answer is perfectly accurate as it matches the information provided in the expected answer. It is complete, addressing all parts of the question, and highly relevant. The phrasing is clear, understandable, and grammatically correct, offering an equally valid way to present the information compared to the expected answer.</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -718,7 +773,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>L'iPhone le moins cher disponible en 128GB est l'**iPhone 11** au prix de **559€**.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -727,7 +782,12 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>The agent's answer is perfectly accurate, complete, relevant, and clear. It identifies the correct iPhone model (iPhone 11) and its price (559€) for the specified storage (128GB), directly matching the expected answer and fully addressing the user's question.</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -743,7 +803,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>L'iPhone 16 offre une autonomie jusqu'à 22h de lecture vidéo, tandis que l'iPhone 13 propose jusqu'à 19h. La différence d'autonomie est donc de 3 heures en faveur de l'iPhone 16.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -752,7 +812,12 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>The agent's answer is perfectly accurate, providing the correct autonomy for both iPhones and calculating the difference accurately. It is complete, addressing all parts of the question. The response is highly relevant and presented with excellent clarity, making it easy to understand. The phrasing is slightly different from the expected answer but conveys the same correct information effectively.</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -768,7 +833,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Oui, si vous êtes encore engagé (avant la fin de votre période de 12 ou 24 mois), des frais de résiliation peuvent s'appliquer. Ces frais sont égaux au montant des mensualités restantes.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -777,7 +842,12 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, clear, and directly addresses all parts of the question asked. It correctly states that fees apply if engaged, specifies they are equal to the remaining monthly payments, and mentions the typical 12 or 24-month periods. While the Expected Answer provides additional helpful context (what happens if not engaged), the question specifically asks 'si je suis engagé' (if I am under contract), which the agent's response fully answers.</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -793,7 +863,8 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Bonjour Jean Bertrand,
+D'après nos informations, votre consommation data pour le mois de **Novembre 2025** est de **3.20 Go**.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -802,7 +873,12 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>The agent's answer is partially accurate regarding the consumed data (3.20 Go) and clear. However, it fails significantly in completeness by omitting the crucial context of the total data allowance (e.g., 'sur votre forfait de 5GB'). Without this information, the user cannot fully understand their data consumption status, making the answer a partial response with a significant missing piece of information. The addition of 'Novembre 2025' for 'ce mois-ci' is also a slight deviation from the expected answer's simplicity, though it might be accurate for the current billing cycle.</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -818,7 +894,18 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Bonjour Jean Bertrand,
+Concernant votre demande sur vos factures, voici le détail :
+Votre **prochaine facture** à régler est celle du mois de **novembre 2025** (facture ID **1**).
+*   **Montant : 9,99€**
+*   **Statut : En attente**
+*   **Date d'échéance : 15 décembre 2025**
+J'attire également votre attention sur une autre facture qui est actuellement en retard :
+*   La facture du mois de **septembre 2025** (facture ID **41**)
+*   **Montant : 9,99€**
+*   **Statut : En retard** (date d'échéance dépassée depuis le 15 octobre 2025)
+Le **montant total** de vos factures en suspens s'élève donc à **19,98€** (9,99€ pour septembre et 9,99€ pour novembre).
+N'hésitez pas si vous avez d'autres questions !</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -827,7 +914,12 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>The agent's answer is perfect. It accurately and completely addresses the user's question about their 'prochaine facture' (next bill), matching the expected amount and due date. Additionally, it provides highly relevant and proactive information about an overdue bill and the total amount due, which significantly enhances the user experience and demonstrates excellent customer support without sacrificing clarity or accuracy.</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -843,7 +935,18 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Bonjour Monsieur Richard,
+Oui, vous avez actuellement **deux tickets de support en cours** dans notre système.
+Voici les détails de vos tickets :
+*   **Ticket ID :** 3
+    *   **Sujet :** Frais de résiliation
+    *   **Statut :** En cours
+    *   **Date de création :** 31 octobre 2025
+*   **Ticket ID :** 4
+    *   **Sujet :** Débit très lent
+    *   **Statut :** En cours
+    *   **Date de création :** 01 novembre 2025
+Nous travaillons sur la résolution de ces deux demandes. N'hésitez pas si vous avez d'autres questions.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -852,7 +955,12 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, relevant, and very clear, providing all essential information requested (number of tickets, IDs, and subjects). It also includes a polite greeting, closing, and creation dates, which are helpful additions. The only minor deviation from the Expected Answer is the absence of the explicit category in parentheses (e.g., 'Résiliation', 'Problème de réseau'), although the 'Sujet' fields largely convey this information. This is a minor omission that does not significantly detract from the answer's completeness or utility.</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -868,7 +976,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Bonjour Jean Bertrand,
+Concernant votre voyage de 2 semaines aux États-Unis, votre forfait actuel **Essentiel 5GB** à **9.99€ par mois** ne comprend pas le roaming dans cette zone. Utiliser votre téléphone aux États-Unis sans option spécifique pourrait entraîner des coûts très élevés.
+Pour éviter cela, nous vous recommandons fortement de souscrire à un **pass international** pour la durée de votre séjour. Vous avez le choix entre :
+*   Un **pass journalier**
+*   Un **pass hebdomadaire**
+Ces pass vous permettront de bénéficier de tarifs avantageux pour vos appels, SMS et données mobiles durant votre voyage de 2 semaines.
+Vous pouvez facilement souscrire et activer le pass de votre choix directement depuis votre **Espace Client** en ligne.
+N'hésitez pas si vous avez d'autres questions !</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -877,7 +992,12 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>The agent's answer is excellent. It accurately identifies the customer's plan, explains the issue with roaming, and provides the correct solution (international passes) with relevant options (daily/weekly). It clearly states where to subscribe (Espace Client), aligning perfectly with the expected answer's guidance. While it doesn't give a specific price for 'combien', it correctly implies that tariffs vary and guides the user to find them, which is the practical and accurate approach for such services. The answer is also clear, well-structured, and includes helpful additional context like the current plan's monthly cost.</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -893,7 +1013,10 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Bonjour Alexandre Martin,
+Oui, vous pouvez tout à fait résilier votre abonnement **sans frais**.
+Votre contrat pour le forfait **Confort 20GB** a débuté le **20 février 2024**. Ce forfait incluait une période d'engagement de 12 mois, qui s'est donc terminée le **20 février 2025**.
+Votre statut actuel est **Actif - Hors engagement**, ce qui confirme que vous êtes libre de résilier votre abonnement à tout moment sans aucuns frais de résiliation.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -902,7 +1025,12 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>The agent's answer is excellent. It directly answers the user's question with a clear 'yes' and confirms the free cancellation. It provides accurate and relevant details, explaining the start date of the contract (20 février 2024), the 12-month engagement period, and the logical end of this period (20 février 2025). This fully supports the conclusion that the user is 'hors engagement' and can cancel without fees. While the expected answer states 'depuis le 14/02/2025', the agent's calculation (20/02/2024 + 12 months = 20/02/2025) is perfectly logical and provides more transparency. The answer is also clear, well-structured, and includes additional helpful information like the specific 'forfait Confort 20GB' and the current 'Actif - Hors engagement' status. It fully addresses all parts of the question with great clarity and completeness.</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -918,7 +1046,8 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Avec un budget de 1000€ et pour une capacité de stockage de 256GB, nous vous recommandons l'**iPhone 14** à 999€.
+Si vous pouviez légèrement dépasser votre budget, l'**iPhone 15** est également disponible en 256GB pour 1099€.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -927,7 +1056,12 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, providing the correct prices for both the iPhone 14 and iPhone 15 at 256GB. It is complete, addressing both the directly affordable option within budget (iPhone 14) and a very close option that slightly exceeds it (iPhone 15), which is helpful. The response is highly relevant to the user's question and is clear and easy to understand. It perfectly matches the expected answer's information.</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -943,7 +1077,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Bonjour Jean Bertrand,
+Merci de nous contacter.
+Concernant votre voyage de 10 jours en Italie, vous serez ravi d'apprendre que vous n'avez **pas besoin de changer de forfait ni de prendre une option supplémentaire** !
+L'Italie faisant partie de l'Union Européenne, vous bénéficiez du "roaming comme à la maison". Cela signifie que vous pouvez utiliser votre forfait actuel **Essentiel 5GB** (incluant 5GB de données mensuelles, appels et SMS illimités) exactement comme si vous étiez en France, sans frais supplémentaires ni restrictions spécifiques (dans la limite d'une utilisation raisonnable).
+Vous pouvez donc partir l'esprit tranquille et utiliser votre téléphone en Italie comme vous le feriez normalement.
+N'hésitez pas si vous avez d'autres questions !</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -952,7 +1091,12 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, complete, relevant, and very clear. It directly answers the user's question about changing their plan or taking an option for their trip to Italy, explaining the 'roaming comme à la maison' policy. It correctly identifies the user's current plan 'Essentiel 5GB' and details its inclusions, aligning perfectly with the expected answer and even offering a more detailed explanation. The tone is also very helpful and reassuring.</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -968,7 +1112,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Oui, vous pouvez bénéficier d'une réduction sur l'achat de l'iPhone 16 en échangeant votre ancien téléphone grâce à notre offre de reprise.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -977,7 +1121,12 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>The agent's answer accurately confirms the possibility of a trade-in discount and is relevant to the question. However, it is incomplete as it doesn't provide the price of the iPhone 16 or crucial actionable information on *how* to proceed with the trade-in (e.g., specific website or contact number), which would be expected from a support chatbot to fully resolve the user's query.</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -993,7 +1142,9 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Les iPhones disponibles avec au moins 48 Mpx de caméra, en version 256GB et pour moins de 1200€ sont :
+*   **iPhone 15** : 1099€
+*   **iPhone 16** : 1149€</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1002,7 +1153,12 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, relevant, and very clear, correctly identifying the iPhone 15 and iPhone 16 as meeting all specified criteria (assuming the hypothetical future context implied by the question and expected answer). It provides the correct prices for these models. However, it is slightly less complete than the expected answer, which also mentions a model (iPhone 17) that has the camera specs but exceeds the budget, providing a more comprehensive understanding of available options to the user.</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1018,7 +1174,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Bonjour Jean Bertrand,
+Je comprends que vous souhaitez connaître le coût supplémentaire pour changer vers un forfait avec plus de data. Actuellement, vous bénéficiez du forfait **Essentiel 5GB** pour **9.99€ par mois**.
+Voici les options de forfaits avec plus de data et les coûts supplémentaires par mois :
+*   **Forfait Confort 20GB** (20 GB de data)
+    *   Prix mensuel : **15.99€**
+    *   Différence de prix : 15.99€ - 9.99€ = **+6.00€ par mois**
+    *   Augmentation de data : **+15 GB** (passant de 5GB à 20GB)
+*   **Forfait Premium 50GB** (50 GB de data)
+    *   Prix mensuel : **24.99€**
+    *   Différence de prix : 24.99€ - 9.99€ = **+15.00€ par mois**
+    *   Augmentation de data : **+45 GB** (passant de 5GB à 50GB)
+*   **Forfait Illimité 100GB** (100 GB de data)
+    *   Prix mensuel : **34.99€**
+    *   Différence de prix : 34.99€ - 9.99€ = **+25.00€ par mois**
+    *   Augmentation de data : **+95 GB** (passant de 5GB à 100GB)
+*   **Forfait Ultra 200GB** (200 GB de data)
+    *   Prix mensuel : **44.99€**
+    *   Différence de prix : 44.99€ - 9.99€ = **+35.00€ par mois**
+    *   Augmentation de data : **+195 GB** (passant de 5GB à 200GB)
+Votre abonnement actuel est **Actif et Engagé** jusqu'au 07 mars 2026. Un changement de forfait peut renouveler votre période d'engagement.
+N'hésitez pas si vous avez d'autres questions ou si vous souhaitez procéder à un changement !</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1027,7 +1203,12 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>The agent's answer is excellent. It accurately identifies the current plan and provides multiple relevant options for upgrading, clearly detailing the price difference and data increase for each. Crucially, it proactively includes important information about the customer's engagement period and how a plan change might affect it, which is vital context for the user. While the expected answer mentioned where and when to change the plan, the agent's comprehensive options and engagement details provide superior value, making it a perfect and highly helpful response.</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1043,7 +1224,8 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Pour la photographie, l'**iPhone 17** est le modèle le plus performant.
+Il est équipé d'une **triple caméra 48 Mpx avec téléobjectif périscopique 5x et capteur LiDAR**, offrant un système photographique capable de capturer des images d'une qualité exceptionnelle dans toutes les conditions d'éclairage.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1052,7 +1234,12 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>The agent's answer correctly identifies the iPhone 17 (following the premise set by the Expected Answer) and provides relevant technical details. However, it is incomplete compared to the Expected Answer, as it fails to mention other excellent alternatives (like the iPhone 16) and, more importantly, omits the crucial advice about budget and specific needs for making a choice. This makes the answer less comprehensive and less helpful for a customer support context.</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1068,7 +1255,9 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hello student, edit me please</t>
+          <t>Oui, vous pouvez utiliser votre iPhone à l'étranger.
+Dans l'Union Européenne, vous bénéficiez du "roaming comme à la maison", ce qui signifie que vous pouvez utiliser votre forfait français sans surcoût, dans la limite de votre contrat.
+Hors Europe, des frais de roaming et des tarifs internationaux s'appliqueront. Pour éviter des surcoûts importants, il est recommandé de désactiver les données mobiles et d'utiliser le WiFi, ou de souscrire à un pass international journalier ou hebdomadaire via votre espace client.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1077,7 +1266,12 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>The agent's answer is accurate, complete, relevant, and very clear. It correctly distinguishes between EU and non-EU usage, explains the 'roaming comme à la maison' principle, and provides excellent practical advice for non-EU travel, including disabling mobile data/using WiFi and subscribing to an international pass via the customer area. The additional detail 'dans la limite de votre contrat' is also a good, accurate clarification. It fully addresses the user's question about using an iPhone abroad without extra cost and provides comprehensive solutions.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final version before langfuse integration
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nous acceptons les paiements par carte bancaire, prélèvement automatique, virement bancaire et PayPal. Le prélèvement automatique est recommandé pour ne jamais manquer une échéance.</t>
+          <t>Nous acceptons les paiements par carte bancaire, prélèvement automatique, virement bancaire et PayPal. Le prélèvement automatique vous garantit de ne jamais manquer une échéance.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, complete, relevant, and clear. It lists all expected payment methods and includes the helpful additional information about direct debit. The minor difference in phrasing ('est recommandé' instead of 'garantit') does not diminish the quality or accuracy of the information provided; in fact, 'recommended' might even be a more appropriate and less absolute claim in a real-world context.</t>
+          <t>The agent's answer is virtually identical to the expected answer. The core information about payment methods is correct and complete. The phrasing 'vous garantit' instead of 'garantit' is a minor, semantically equivalent difference and does not affect accuracy, completeness, relevance, or clarity. It fully answers the question and provides helpful information.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vous pouvez consulter vos factures en vous connectant à votre espace client sur notre site web ou via l'application mobile. Toutes vos factures sont disponibles dans la section 'Mes factures' pendant 24 mois.</t>
+          <t>Vous pouvez consulter vos factures en ligne en vous connectant à votre espace client sur notre site web ou via l'application mobile. Toutes vos factures sont disponibles dans la section 'Mes factures' pendant 24 mois.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The agent's answer is virtually identical to the expected answer. It provides correct, complete, relevant, and clear information on how to consult invoices online. The only minor difference is 'notre site web' instead of 'le site web', which is equally accurate and appropriate in the context of a company's chatbot.</t>
+          <t>The agent's answer is virtually identical to the expected answer. It provides accurate, complete, relevant, and clear instructions on how to view invoices online, including where to log in, the platforms available, the section to find them, and the retention period. Minor phrasing differences ('sur le site web' vs 'sur notre site web', 'Toutes les factures' vs 'Toutes vos factures') do not impact the core information or clarity, aligning perfectly with a lenient evaluation.</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Oui, TelecomPlus propose des forfaits famille qui permettent de partager un pool de données entre plusieurs lignes. Pour plus d'informations sur nos offres multi-lignes, vous pouvez contacter notre service client.</t>
+          <t>Bonjour !
+Je comprends votre question concernant le partage de votre forfait data avec votre famille.
+D'après les informations disponibles dans notre système concernant les forfaits TelecomPlus, les offres que nous proposons actuellement, telles que **Essentiel 5GB**, **Confort 20GB**, **Premium 50GB**, **Illimité 100GB** et **Ultra 200GB**, sont des forfaits individuels.
+Ces forfaits sont conçus pour une utilisation par un seul utilisateur et n'incluent pas, en standard, de fonctionnalité de partage de données directement entre différentes lignes ou avec d'autres membres de la famille.
+Chaque forfait dispose de sa propre allocation de données mensuelles pour l'abonné principal :
+*   **Essentiel 5GB** : 5 Go
+*   **Confort 20GB** : 20 Go
+*   **Premium 50GB** : 50 Go
+*   **Illimité 100GB** : 100 Go
+*   **Ultra 200GB** : 200 Go
+Si vous souhaitez que les membres de votre famille bénéficient également d'un forfait data, nous vous invitons à consulter nos différentes offres afin de trouver le forfait le plus adapté à leurs besoins.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -542,11 +552,11 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>The agent's answer is almost identical to the expected answer. It is accurate, complete, relevant, and very clear. It confirms the possibility of sharing data through family plans and correctly advises contacting customer service for more details on multi-line offers. The slight rephrasing and inclusion of 'TelecomPlus' do not detract from its quality.</t>
+          <t>The agent's answer correctly identifies that the specific listed plans are individual and do not support data sharing. However, the expected answer indicates that the company *does* offer family plans that allow data sharing. The agent completely misses this crucial information, making its answer partially correct for individual plans but misleading regarding the overall possibility of data sharing within the company's offerings. This omission could lead the customer to believe sharing is impossible, contradicting the expected solution.</t>
         </is>
       </c>
     </row>
@@ -563,7 +573,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Le roaming international est généralement activé par défaut. Vous pouvez vérifier son statut dans votre espace client en ligne ou en appelant le service client. N'oubliez pas de vérifier les tarifs applicables avant de voyager.</t>
+          <t>Le roaming international est généralement activé par défaut. Vous pouvez vérifier son statut et l'activer si nécessaire dans votre espace client ou en appelant le service client. Nous vous recommandons de vérifier les tarifs applicables avant de voyager.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -576,7 +586,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>The agent's answer is virtually identical to the expected answer, providing accurate, complete, and relevant information with excellent clarity. The minor phrasing differences ('espace client en ligne' vs 'espace client', 'N'oubliez pas' vs 'Pensez à', 'tarifs applicables' vs 'tarifs') do not detract from its quality and, in some cases, slightly enhance it.</t>
+          <t>The agent's answer is accurate, complete, and clearly addresses the customer's question. It matches the core information in the expected answer and even improves upon it by explicitly stating 'et l'activer si nécessaire' in the suggested steps, directly answering the 'How to activate' part. All recommendations are helpful and actionable. Minor phrasing differences do not impact the score, as per the leniency guidelines.</t>
         </is>
       </c>
     </row>
@@ -593,7 +603,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dans l'Union Européenne, vous bénéficiez du "roaming comme à la maison", ce qui signifie que vous pouvez utiliser votre forfait français sans surcoût dans les pays de l'UE, selon les limites de votre contrat.</t>
+          <t>Dans l'Union Européenne, vous bénéficiez du 'roaming comme à la maison'. Cela signifie que vous pouvez utiliser votre forfait français sans surcoût dans les pays de l'UE, selon les limites de votre contrat.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -606,7 +616,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, complete, relevant, and very clear. It perfectly matches the expected answer, providing all necessary information about 'roaming comme à la maison' within the EU, including the no surcharges and contract limits conditions. The slight difference ('ce qui signifie que') actually enhances clarity without changing the core message or adding redundancy.</t>
+          <t>The agent's answer is practically identical to the expected answer, providing accurate, complete, and clear information about roaming tariffs in the EU. The slight rephrasing ('Cela signifie que') adds clarity without altering the core message, which is a positive under lenient evaluation.</t>
         </is>
       </c>
     </row>
@@ -623,7 +633,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Si vous avez oublié votre mot de passe, cliquez sur 'Mot de passe oublié' sur la page de connexion de votre espace client. Vous recevrez alors un lien de réinitialisation par email ou SMS, suivez les instructions pour créer un nouveau mot de passe.</t>
+          <t>Si vous avez oublié votre mot de passe, cliquez sur 'Mot de passe oublié' sur la page de connexion de votre espace client. Vous recevrez un lien de réinitialisation par email ou SMS. Suivez les instructions pour créer un nouveau mot de passe.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -636,7 +646,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>The agent's answer is excellent. It is accurate, complete, relevant, and very clear. It provides the exact information needed, matching the expected answer almost perfectly, with a slightly more natural conversational opening.</t>
+          <t>The agent's answer is almost identical to the expected answer. It accurately provides all the core information, is complete, relevant, and very clear. The slight phrasing difference ('de votre espace client') is a minor addition that does not detract from the answer, and in fact, makes it slightly more specific and helpful. This perfectly aligns with the lenient evaluation criteria.</t>
         </is>
       </c>
     </row>
@@ -653,7 +663,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Les paramètres MMS sont généralement configurés automatiquement. Si ce n'est pas le cas, vous pouvez vous rendre dans Réglages &gt; Réseau mobile &gt; Noms des points d'accès et ajouter la configuration disponible sur notre site web.</t>
+          <t>Pour configurer vos MMS, les paramètres sont généralement configurés automatiquement. Si ce n'est pas le cas, vous pouvez vous rendre dans Réglages &gt; Réseau mobile &gt; Noms des points d'accès et ajouter la configuration disponible sur notre site web.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -666,7 +676,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>The agent's answer is virtually identical to the expected answer, providing accurate, complete, relevant, and clear instructions. The minor stylistic differences ('vous pouvez vous rendre' vs 'rendez-vous' and 'site web' vs 'site') do not impact the quality or understanding of the response.</t>
+          <t>The agent's answer is virtually identical to the expected answer, providing the same core information and steps. It accurately states that MMS settings are usually automatic, and provides the exact navigation path (Réglages &gt; Réseau mobile &gt; Noms des points d'accès) along with the advice to find the configuration on the website. All evaluation criteria (Accuracy, Completeness, Relevance, Clarity) are met fully. Minor phrasing differences ('site web' vs 'site') do not impact the score as per the lenient guidelines.</t>
         </is>
       </c>
     </row>
@@ -683,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Le prix de l'iPhone 15 en version 256GB est de **1099€**.</t>
+          <t>Le prix de l'iPhone 15 en version 256GB est de 1099€.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -696,7 +706,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, complete, relevant, and very clear. It directly addresses the question and provides the correct price, matching the expected answer's information perfectly, with a slightly different but equally valid phrasing.</t>
+          <t>The agent's answer is perfectly accurate, complete, relevant, and clear. It provides the exact core information (the price of the iPhone 15 256GB) as expected. The phrasing difference is minor and does not impact the quality or understanding of the answer, fully aligning with the lenient evaluation criteria.</t>
         </is>
       </c>
     </row>
@@ -726,7 +736,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>The agent's answer is identical to the expected answer. It is factually accurate, directly answers the question, is complete, and clearly understandable. The iPhone 15 series was indeed released in 2023.</t>
+          <t>The agent's answer is identical to the expected answer, providing the correct iPhone model (iPhone 15) and year of commercialization (2023). It is accurate, complete, relevant, and clear, fully meeting the customer's request.</t>
         </is>
       </c>
     </row>
@@ -756,7 +766,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>The agent's answer is perfectly accurate as it matches the information provided in the expected answer. It is complete, addressing all parts of the question, and highly relevant. The phrasing is clear, understandable, and grammatically correct, offering an equally valid way to present the information compared to the expected answer.</t>
+          <t>The agent's answer provides the exact same core information (list of colors) as the expected answer. The phrasing is slightly different but conveys the identical meaning and is perfectly clear and accurate. It fully answers the customer's question effectively.</t>
         </is>
       </c>
     </row>
@@ -786,7 +796,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>The agent's answer is perfectly accurate, complete, relevant, and clear. It identifies the correct iPhone model (iPhone 11) and its price (559€) for the specified storage (128GB), directly matching the expected answer and fully addressing the user's question.</t>
+          <t>The agent's answer is perfectly accurate, complete, relevant, and clear. It provides the exact model (iPhone 11) and price (559€) as expected, directly answering the customer's question about the cheapest 128GB iPhone.</t>
         </is>
       </c>
     </row>
@@ -803,7 +813,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>L'iPhone 16 offre une autonomie jusqu'à 22h de lecture vidéo, tandis que l'iPhone 13 propose jusqu'à 19h. La différence d'autonomie est donc de 3 heures en faveur de l'iPhone 16.</t>
+          <t>L'iPhone 16 offre une autonomie de lecture vidéo jusqu'à 22h, tandis que l'iPhone 13 propose une autonomie jusqu'à 19h. L'iPhone 16 a donc une autonomie supérieure de 3 heures par rapport à l'iPhone 13.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -816,7 +826,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>The agent's answer is perfectly accurate, providing the correct autonomy for both iPhones and calculating the difference accurately. It is complete, addressing all parts of the question. The response is highly relevant and presented with excellent clarity, making it easy to understand. The phrasing is slightly different from the expected answer but conveys the same correct information effectively.</t>
+          <t>The agent's answer provides the exact same core information as the expected answer. It correctly states the battery life for both iPhones and accurately calculates the 3-hour difference. The phrasing is slightly different but conveys the identical and correct information clearly, fully, and relevantly to the customer. This fully meets all evaluation criteria, especially given the lenient instructions.</t>
         </is>
       </c>
     </row>
@@ -833,7 +843,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Oui, si vous êtes encore engagé (avant la fin de votre période de 12 ou 24 mois), des frais de résiliation peuvent s'appliquer. Ces frais sont égaux au montant des mensualités restantes.</t>
+          <t>Oui, si vous êtes encore engagé, des frais de résiliation peuvent s'appliquer, égaux au montant des mensualités restantes. En revanche, si vous êtes hors période d'engagement (après 12 ou 24 mois), la résiliation est gratuite.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -846,7 +856,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, clear, and directly addresses all parts of the question asked. It correctly states that fees apply if engaged, specifies they are equal to the remaining monthly payments, and mentions the typical 12 or 24-month periods. While the Expected Answer provides additional helpful context (what happens if not engaged), the question specifically asks 'si je suis engagé' (if I am under contract), which the agent's response fully answers.</t>
+          <t>The agent's answer is accurate, complete, relevant, and clear. It provides the core information identical to the expected answer, explaining that fees apply if engaged (equal to remaining monthly payments) and that it's free if out of commitment (after 12 or 24 months). The phrasing is slightly different but conveys the exact same helpful information to the customer without any omissions or inaccuracies. It directly answers 'Oui' to the question, which is appropriate.</t>
         </is>
       </c>
     </row>
@@ -864,7 +874,9 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>Bonjour Jean Bertrand,
-D'après nos informations, votre consommation data pour le mois de **Novembre 2025** est de **3.20 Go**.</t>
+Pour ce mois-ci (Novembre 2025), votre consommation data est de **3.20 Go**.
+Vous avez donc utilisé 3.20 Go sur votre forfait **Essentiel 5GB** qui inclut un total de **5 Go** de data par mois.
+Il vous reste ainsi **1.80 Go** de data à utiliser pour le mois de Novembre 2025.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -873,11 +885,11 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>The agent's answer is partially accurate regarding the consumed data (3.20 Go) and clear. However, it fails significantly in completeness by omitting the crucial context of the total data allowance (e.g., 'sur votre forfait de 5GB'). Without this information, the user cannot fully understand their data consumption status, making the answer a partial response with a significant missing piece of information. The addition of 'Novembre 2025' for 'ce mois-ci' is also a slight deviation from the expected answer's simplicity, though it might be accurate for the current billing cycle.</t>
+          <t>The agent's answer is accurate, complete, relevant, and clear. It directly answers the customer's question about data consumption (3.20 Go) and provides the context of their plan (5 Go). Furthermore, it proactively offers additional helpful information by calculating the remaining data (1.80 Go), which is considered a positive in this lenient evaluation. The agent even greets the customer by name. All core information is correct and well-presented.</t>
         </is>
       </c>
     </row>
@@ -895,17 +907,11 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>Bonjour Jean Bertrand,
-Concernant votre demande sur vos factures, voici le détail :
-Votre **prochaine facture** à régler est celle du mois de **novembre 2025** (facture ID **1**).
-*   **Montant : 9,99€**
-*   **Statut : En attente**
-*   **Date d'échéance : 15 décembre 2025**
-J'attire également votre attention sur une autre facture qui est actuellement en retard :
-*   La facture du mois de **septembre 2025** (facture ID **41**)
-*   **Montant : 9,99€**
-*   **Statut : En retard** (date d'échéance dépassée depuis le 15 octobre 2025)
-Le **montant total** de vos factures en suspens s'élève donc à **19,98€** (9,99€ pour septembre et 9,99€ pour novembre).
-N'hésitez pas si vous avez d'autres questions !</t>
+Voici les détails concernant votre prochaine facture :
+*   **Montant de votre prochaine facture :** **9.99 €**
+*   **Mois concerné :** Novembre 2025
+*   **Date d'échéance :** 15 décembre 2025
+Cette facture (ID : 1) est actuellement "En attente" de paiement.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -918,7 +924,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>The agent's answer is perfect. It accurately and completely addresses the user's question about their 'prochaine facture' (next bill), matching the expected amount and due date. Additionally, it provides highly relevant and proactive information about an overdue bill and the total amount due, which significantly enhances the user experience and demonstrates excellent customer support without sacrificing clarity or accuracy.</t>
+          <t>The agent accurately provides the core information requested: the amount of the next bill (9.99€) and its due date (15 décembre 2025). The agent also provides additional helpful and relevant details such as the month concerned, a bill ID, and the payment status, which is a bonus according to the lenient criteria. The answer is clear and easy to understand.</t>
         </is>
       </c>
     </row>
@@ -936,17 +942,16 @@
       <c r="C17" t="inlineStr">
         <is>
           <t>Bonjour Monsieur Richard,
-Oui, vous avez actuellement **deux tickets de support en cours** dans notre système.
-Voici les détails de vos tickets :
-*   **Ticket ID :** 3
+Oui, j'ai trouvé **deux tickets de support en cours** associés à votre compte dans notre système :
+*   **ID du ticket : 3**
     *   **Sujet :** Frais de résiliation
     *   **Statut :** En cours
-    *   **Date de création :** 31 octobre 2025
-*   **Ticket ID :** 4
+    *   **Date de création :** 2025-10-31
+*   **ID du ticket : 4**
     *   **Sujet :** Débit très lent
     *   **Statut :** En cours
-    *   **Date de création :** 01 novembre 2025
-Nous travaillons sur la résolution de ces deux demandes. N'hésitez pas si vous avez d'autres questions.</t>
+    *   **Date de création :** 2025-11-01
+Nous restons à votre disposition pour toute information complémentaire.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -955,11 +960,11 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, relevant, and very clear, providing all essential information requested (number of tickets, IDs, and subjects). It also includes a polite greeting, closing, and creation dates, which are helpful additions. The only minor deviation from the Expected Answer is the absence of the explicit category in parentheses (e.g., 'Résiliation', 'Problème de réseau'), although the 'Sujet' fields largely convey this information. This is a minor omission that does not significantly detract from the answer's completeness or utility.</t>
+          <t>The agent correctly identifies that there are two tickets in progress and provides the exact ID and subject for each, matching the expected answer. It also adds helpful details like status and creation date, which is considered a positive under the lenient evaluation criteria.</t>
         </is>
       </c>
     </row>
@@ -977,13 +982,15 @@
       <c r="C18" t="inlineStr">
         <is>
           <t>Bonjour Jean Bertrand,
-Concernant votre voyage de 2 semaines aux États-Unis, votre forfait actuel **Essentiel 5GB** à **9.99€ par mois** ne comprend pas le roaming dans cette zone. Utiliser votre téléphone aux États-Unis sans option spécifique pourrait entraîner des coûts très élevés.
-Pour éviter cela, nous vous recommandons fortement de souscrire à un **pass international** pour la durée de votre séjour. Vous avez le choix entre :
-*   Un **pass journalier**
-*   Un **pass hebdomadaire**
-Ces pass vous permettront de bénéficier de tarifs avantageux pour vos appels, SMS et données mobiles durant votre voyage de 2 semaines.
-Vous pouvez facilement souscrire et activer le pass de votre choix directement depuis votre **Espace Client** en ligne.
-N'hésitez pas si vous avez d'autres questions !</t>
+Concernant votre voyage de 2 semaines aux États-Unis, voici les informations importantes concernant l'utilisation de votre forfait.
+Vous disposez actuellement du **Forfait Essentiel 5GB**, qui inclut **5 Go de données mobiles** par mois pour un tarif de 9.99€.
+Étant donné que les États-Unis ne font pas partie de l'Union Européenne, le "roaming comme à la maison" ne s'applique pas. Des frais de roaming international peuvent donc être appliqués si vous utilisez votre forfait (appels, SMS, internet mobile) sur place.
+Pour éviter des frais inattendus lors de votre séjour aux États-Unis, nous vous recommandons les options suivantes :
+*   **Désactiver les données mobiles** sur votre téléphone et privilégier l'utilisation du **Wi-Fi** lorsque disponible.
+*   **Souscrire à un pass international** journalier ou hebdomadaire. Ces pass sont spécifiquement conçus pour les voyages hors Europe et vous permettent de maîtriser votre budget. Vous pouvez consulter les différentes options et tarifs, ainsi que souscrire à un pass, directement depuis votre **espace client en ligne**.
+Les tarifs exacts pour les appels, SMS et données mobiles aux États-Unis sans pass dépendent de votre consommation et sont disponibles en détail dans votre espace client.
+Pour obtenir des informations tarifaires plus précises ou pour souscrire à un pass international avant votre départ, n'hésitez pas à contacter notre service client au **3900** (appel gratuit, disponible 7j/7 de 8h à 20h) ou à consulter votre **espace client** sur www.telecomplus.fr/mon-compte.
+Nous vous souhaitons un excellent voyage aux États-Unis !</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -996,7 +1003,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>The agent's answer is excellent. It accurately identifies the customer's plan, explains the issue with roaming, and provides the correct solution (international passes) with relevant options (daily/weekly). It clearly states where to subscribe (Espace Client), aligning perfectly with the expected answer's guidance. While it doesn't give a specific price for 'combien', it correctly implies that tariffs vary and guides the user to find them, which is the practical and accurate approach for such services. The answer is also clear, well-structured, and includes helpful additional context like the current plan's monthly cost.</t>
+          <t>The agent's answer is excellent. It accurately identifies the customer's plan, correctly explains roaming outside the EU, recommends international passes (daily/weekly) and advises consulting the customer space for tariffs, exactly as the expected answer does. Furthermore, it provides valuable additional context, practical tips (Wi-Fi, disabling data), and clear contact information, which is highly helpful to the customer. It completely fulfills and even exceeds the 'Expected Answer' while remaining perfectly accurate, complete, relevant, and clear.</t>
         </is>
       </c>
     </row>
@@ -1014,9 +1021,10 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>Bonjour Alexandre Martin,
-Oui, vous pouvez tout à fait résilier votre abonnement **sans frais**.
-Votre contrat pour le forfait **Confort 20GB** a débuté le **20 février 2024**. Ce forfait incluait une période d'engagement de 12 mois, qui s'est donc terminée le **20 février 2025**.
-Votre statut actuel est **Actif - Hors engagement**, ce qui confirme que vous êtes libre de résilier votre abonnement à tout moment sans aucuns frais de résiliation.</t>
+Concernant votre question sur la résiliation de votre abonnement, je peux vous confirmer que votre forfait actuel **Confort 20GB** est en statut **Actif - Hors engagement**.
+Votre contrat a débuté le **20 février 2024**.
+Étant donné que vous êtes actuellement **hors période d'engagement**, vous pouvez **tout à fait résilier votre abonnement sans aucuns frais**.
+Pour procéder à la résiliation, vous pouvez vous rendre dans votre **Espace Client** en ligne ou contacter notre service client au **3900**. La résiliation prendra effet à la fin de votre cycle de facturation actuel.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1029,7 +1037,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>The agent's answer is excellent. It directly answers the user's question with a clear 'yes' and confirms the free cancellation. It provides accurate and relevant details, explaining the start date of the contract (20 février 2024), the 12-month engagement period, and the logical end of this period (20 février 2025). This fully supports the conclusion that the user is 'hors engagement' and can cancel without fees. While the expected answer states 'depuis le 14/02/2025', the agent's calculation (20/02/2024 + 12 months = 20/02/2025) is perfectly logical and provides more transparency. The answer is also clear, well-structured, and includes additional helpful information like the specific 'forfait Confort 20GB' and the current 'Actif - Hors engagement' status. It fully addresses all parts of the question with great clarity and completeness.</t>
+          <t>The agent accurately confirms that the customer can cancel their subscription without fees, which is the core of the expected answer. It correctly states the contract start date and confirms the 'hors engagement' status. Furthermore, it provides helpful additional information on how to proceed with the cancellation (Espace Client, phone number) and clarifies when the cancellation takes effect, which is considered a positive under the lenient evaluation criteria.</t>
         </is>
       </c>
     </row>
@@ -1046,8 +1054,8 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Avec un budget de 1000€ et pour une capacité de stockage de 256GB, nous vous recommandons l'**iPhone 14** à 999€.
-Si vous pouviez légèrement dépasser votre budget, l'**iPhone 15** est également disponible en 256GB pour 1099€.</t>
+          <t>Avec un budget de 1000€ pour un iPhone en version 256GB, nous vous recommandons l'**iPhone 14** à 999€.
+Si vous pouviez légèrement ajuster votre budget, l'**iPhone 15** en 256GB est disponible pour 1099€.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1060,7 +1068,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, providing the correct prices for both the iPhone 14 and iPhone 15 at 256GB. It is complete, addressing both the directly affordable option within budget (iPhone 14) and a very close option that slightly exceeds it (iPhone 15), which is helpful. The response is highly relevant to the user's question and is clear and easy to understand. It perfectly matches the expected answer's information.</t>
+          <t>The agent's answer is accurate, complete, relevant, and clear. It correctly identifies the iPhone 14 (256GB) at 999€ as an option within budget and also provides the iPhone 15 (256GB) at 1099€ as an alternative just above the budget, matching the expected answer perfectly. This is extremely helpful to the customer.</t>
         </is>
       </c>
     </row>
@@ -1077,11 +1085,36 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bonjour Jean Bertrand,
-Merci de nous contacter.
-Concernant votre voyage de 10 jours en Italie, vous serez ravi d'apprendre que vous n'avez **pas besoin de changer de forfait ni de prendre une option supplémentaire** !
-L'Italie faisant partie de l'Union Européenne, vous bénéficiez du "roaming comme à la maison". Cela signifie que vous pouvez utiliser votre forfait actuel **Essentiel 5GB** (incluant 5GB de données mensuelles, appels et SMS illimités) exactement comme si vous étiez en France, sans frais supplémentaires ni restrictions spécifiques (dans la limite d'une utilisation raisonnable).
-Vous pouvez donc partir l'esprit tranquille et utiliser votre téléphone en Italie comme vous le feriez normalement.
+          <t>Bonjour Monsieur Bertrand,
+Je comprends que vous préparez votre voyage en Italie et vous vous interrogez sur l'utilisation de votre forfait.
+Bonne nouvelle ! L'Italie fait partie de l'Union Européenne, ce qui signifie que vous bénéficiez du **"roaming comme à la maison"**.
+Cela signifie que vous pouvez utiliser votre forfait actuel en Italie comme si vous étiez en France, sans frais supplémentaires.
+### Votre Forfait Actuel
+*   **Forfait :** Essentiel 5GB
+*   **Données mobiles :** **5 Go** par mois
+*   **Appels et SMS :** Illimités
+*   **Prix mensuel :** 9.99 €
+Vous pourrez utiliser vos **5 Go de données mobiles**, ainsi que les appels et SMS illimités inclus dans votre forfait, sans surcoût pendant votre séjour de 10 jours en Italie.
+### Recommandation pour votre voyage
+Pour un séjour de 10 jours, **5 Go** peuvent être suffisants pour une utilisation modérée (consultation d'e-mails, navigation légère, messagerie instantanée). Cependant, si vous prévoyez d'utiliser intensivement internet (streaming vidéo, GPS fréquent, appels vidéo), il est possible que ces 5 Go soient un peu justes.
+Je vous recommande de surveiller votre consommation de données via votre Espace Client ou l'application TelecomPlus pour vous assurer que vous ne dépassez pas votre allocation.
+### Options si vous avez besoin de plus de données
+Si vous estimez que 5 Go ne seront pas suffisants pour votre séjour, vous avez la possibilité de changer de forfait pour bénéficier de plus de données. Voici les forfaits supérieurs disponibles et les différences de prix et de données :
+*   **Forfait Confort 20GB**
+    *   **Données :** 20 Go (**+15 Go** par rapport à votre forfait actuel)
+    *   **Prix mensuel :** 15.99 € (**+6.00 €** par mois par rapport à votre forfait actuel)
+*   **Forfait Premium 50GB**
+    *   **Données :** 50 Go (**+45 Go** par rapport à votre forfait actuel)
+    *   **Prix mensuel :** 24.99 € (**+15.00 €** par mois par rapport à votre forfait actuel)
+*   **Forfait Illimité 100GB**
+    *   **Données :** 100 Go (**+95 Go** par rapport à votre forfait actuel)
+    *   **Prix mensuel :** 34.99 € (**+25.00 €** par mois par rapport à votre forfait actuel)
+*   **Forfait Ultra 200GB**
+    *   **Données :** 200 Go (**+195 Go** par rapport à votre forfait actuel)
+    *   **Prix mensuel :** 44.99 € (**+35.00 €** par mois par rapport à votre forfait actuel)
+### Comment changer de forfait ?
+Vous pouvez modifier votre forfait directement depuis votre **Espace Client en ligne** ou en appelant le **3900**. Le changement prendra effet au **début de votre prochain cycle de facturation**.
+Actuellement, votre forfait est **Actif et Engagé** jusqu'au 07/03/2026. Changer pour un forfait supérieur n'affectera pas votre engagement mais le mettra à jour avec les nouvelles conditions.
 N'hésitez pas si vous avez d'autres questions !</t>
         </is>
       </c>
@@ -1095,7 +1128,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, complete, relevant, and very clear. It directly answers the user's question about changing their plan or taking an option for their trip to Italy, explaining the 'roaming comme à la maison' policy. It correctly identifies the user's current plan 'Essentiel 5GB' and details its inclusions, aligning perfectly with the expected answer and even offering a more detailed explanation. The tone is also very helpful and reassuring.</t>
+          <t>The agent's answer is excellent. It correctly identifies that roaming in Italy is included ('roaming comme à la maison') and that no extra option is needed, directly answering the core question. It goes above and beyond by detailing the customer's current plan, providing practical advice on data consumption for a 10-day trip, and proactively offering clear options for upgrading the plan if the customer feels 5GB won't be enough. The instructions on how to change the plan and details about the engagement are also very helpful. This response is accurate, complete, highly relevant, and very clear.</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1145,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Oui, vous pouvez bénéficier d'une réduction sur l'achat de l'iPhone 16 en échangeant votre ancien téléphone grâce à notre offre de reprise.</t>
+          <t>Oui, absolument ! Chez TelecomPlus, vous pouvez échanger votre ancien téléphone et bénéficier d'une réduction sur l'achat de votre nouvel iPhone 16.
+Le prix de l'iPhone 16 commence à 1019€ pour le modèle 128GB.
+Pour connaître le montant de la réduction liée à la reprise de votre ancien téléphone et pour finaliser votre achat, vous pouvez :
+*   Nous appeler au **3900** (appel gratuit).
+*   Vous rendre dans l'une de nos **boutiques** pour une évaluation.
+*   Commander en ligne sur **www.telecomplus.fr**.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1121,11 +1159,11 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>The agent's answer accurately confirms the possibility of a trade-in discount and is relevant to the question. However, it is incomplete as it doesn't provide the price of the iPhone 16 or crucial actionable information on *how* to proceed with the trade-in (e.g., specific website or contact number), which would be expected from a support chatbot to fully resolve the user's query.</t>
+          <t>The agent's answer is excellent. It directly confirms that a reduction is possible through trade-in, provides the correct starting price for the iPhone 16, and offers clear, actionable steps for the customer to proceed (phone, in-store, online). It aligns perfectly with the expected answer's core information and even adds an additional helpful option (visiting a store), which is a positive under lenient evaluation. All criteria (accuracy, completeness, relevance, clarity) are met.</t>
         </is>
       </c>
     </row>
@@ -1142,9 +1180,10 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Les iPhones disponibles avec au moins 48 Mpx de caméra, en version 256GB et pour moins de 1200€ sont :
-*   **iPhone 15** : 1099€
-*   **iPhone 16** : 1149€</t>
+          <t>Pour un iPhone avec au moins 48 Mpx de caméra et 256GB de stockage pour moins de 1200€, vous avez les options suivantes :
+*   **iPhone 15 (256GB)** à 1099€. Il dispose d'une double caméra 48 Mpx (principal) et 12 Mpx (ultra grand-angle).
+*   **iPhone 16 (256GB)** à 1149€. Il est équipé d'un système de caméra Fusion 48 Mpx avec ultra grand-angle amélioré.
+L'iPhone 17 propose également une triple caméra 48 Mpx, mais son modèle 256GB est à 1299€, ce qui dépasse votre budget de 1200€.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1153,11 +1192,11 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, relevant, and very clear, correctly identifying the iPhone 15 and iPhone 16 as meeting all specified criteria (assuming the hypothetical future context implied by the question and expected answer). It provides the correct prices for these models. However, it is slightly less complete than the expected answer, which also mentions a model (iPhone 17) that has the camera specs but exceeds the budget, providing a more comprehensive understanding of available options to the user.</t>
+          <t>The agent's answer is accurate, complete, relevant, and clear. It correctly identifies the iPhone 15 and 16 as fitting the criteria (model, storage, camera Mpx, and price). It also correctly notes that the iPhone 17 exceeds the budget, providing the correct price for it. The additional details about the camera systems are helpful and do not detract from the core answer.</t>
         </is>
       </c>
     </row>
@@ -1174,27 +1213,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bonjour Jean Bertrand,
-Je comprends que vous souhaitez connaître le coût supplémentaire pour changer vers un forfait avec plus de data. Actuellement, vous bénéficiez du forfait **Essentiel 5GB** pour **9.99€ par mois**.
-Voici les options de forfaits avec plus de data et les coûts supplémentaires par mois :
-*   **Forfait Confort 20GB** (20 GB de data)
-    *   Prix mensuel : **15.99€**
-    *   Différence de prix : 15.99€ - 9.99€ = **+6.00€ par mois**
-    *   Augmentation de data : **+15 GB** (passant de 5GB à 20GB)
-*   **Forfait Premium 50GB** (50 GB de data)
-    *   Prix mensuel : **24.99€**
-    *   Différence de prix : 24.99€ - 9.99€ = **+15.00€ par mois**
-    *   Augmentation de data : **+45 GB** (passant de 5GB à 50GB)
-*   **Forfait Illimité 100GB** (100 GB de data)
-    *   Prix mensuel : **34.99€**
-    *   Différence de prix : 34.99€ - 9.99€ = **+25.00€ par mois**
-    *   Augmentation de data : **+95 GB** (passant de 5GB à 100GB)
-*   **Forfait Ultra 200GB** (200 GB de data)
-    *   Prix mensuel : **44.99€**
-    *   Différence de prix : 44.99€ - 9.99€ = **+35.00€ par mois**
-    *   Augmentation de data : **+195 GB** (passant de 5GB à 200GB)
-Votre abonnement actuel est **Actif et Engagé** jusqu'au 07 mars 2026. Un changement de forfait peut renouveler votre période d'engagement.
-N'hésitez pas si vous avez d'autres questions ou si vous souhaitez procéder à un changement !</t>
+          <t>Bonjour M. Bertrand,
+Vous avez actuellement le forfait **Essentiel 5GB** pour un montant de **9.99€** par mois.
+Si vous souhaitez changer pour un forfait avec plus de data, voici les options disponibles et le coût supplémentaire par mois que cela représenterait :
+*   **Forfait Confort 20GB**
+    *   Vous passeriez à **20 Go** de data par mois (soit **15 Go de plus**).
+    *   Le prix mensuel serait de **15.99€**, soit **6.00€ de plus** par mois.
+*   **Forfait Premium 50GB**
+    *   Vous passeriez à **50 Go** de data par mois (soit **45 Go de plus**).
+    *   Le prix mensuel serait de **24.99€**, soit **15.00€ de plus** par mois.
+*   **Forfait Illimité 100GB**
+    *   Vous passeriez à **100 Go** de data par mois (soit **95 Go de plus**).
+    *   Le prix mensuel serait de **34.99€**, soit **25.00€ de plus** par mois.
+*   **Forfait Ultra 200GB**
+    *   Vous passeriez à **200 Go** de data par mois (soit **195 Go de plus**).
+    *   Le prix mensuel serait de **44.99€**, soit **35.00€ de plus** par mois.
+Pour changer de forfait, vous pouvez le faire facilement depuis votre Espace Client en ligne ou en appelant le 3900. Le changement prendra effet au début de votre prochain cycle de facturation.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1207,7 +1241,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>The agent's answer is excellent. It accurately identifies the current plan and provides multiple relevant options for upgrading, clearly detailing the price difference and data increase for each. Crucially, it proactively includes important information about the customer's engagement period and how a plan change might affect it, which is vital context for the user. While the expected answer mentioned where and when to change the plan, the agent's comprehensive options and engagement details provide superior value, making it a perfect and highly helpful response.</t>
+          <t>The agent's answer is excellent. It accurately identifies the customer's current plan and provides not just one, but multiple options for plans with more data, along with the precise additional cost for each. This is more comprehensive than the expected answer and very helpful for the customer. It also clearly outlines how to change the plan and when the change will be effective. All information is accurate, complete, relevant, and clearly presented, exceeding expectations.</t>
         </is>
       </c>
     </row>
@@ -1224,8 +1258,8 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pour la photographie, l'**iPhone 17** est le modèle le plus performant.
-Il est équipé d'une **triple caméra 48 Mpx avec téléobjectif périscopique 5x et capteur LiDAR**, offrant un système photographique capable de capturer des images d'une qualité exceptionnelle dans toutes les conditions d'éclairage.</t>
+          <t>Pour la photographie, l'**iPhone 17** est le meilleur choix. Il dispose d'une triple caméra 48 Mpx avec téléobjectif périscopique 5x et capteur LiDAR, permettant de capturer des images d'une qualité exceptionnelle dans toutes les conditions d'éclairage.
+Une excellente alternative est l'**iPhone 16**, qui propose également un système de caméra Fusion 48 Mpx avec ultra grand-angle amélioré.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1234,11 +1268,11 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>The agent's answer correctly identifies the iPhone 17 (following the premise set by the Expected Answer) and provides relevant technical details. However, it is incomplete compared to the Expected Answer, as it fails to mention other excellent alternatives (like the iPhone 16) and, more importantly, omits the crucial advice about budget and specific needs for making a choice. This makes the answer less comprehensive and less helpful for a customer support context.</t>
+          <t>The agent provides an excellent and comprehensive answer. It correctly identifies the best iPhone (17) and a strong alternative (16), along with accurate and relevant technical specifications for both. The information is clear and directly addresses the customer's question effectively, even providing slightly more detail for the iPhone 16 than expected, which is a bonus according to the lenient criteria. The core information is perfectly aligned with the expected answer.</t>
         </is>
       </c>
     </row>
@@ -1256,8 +1290,9 @@
       <c r="C26" t="inlineStr">
         <is>
           <t>Oui, vous pouvez utiliser votre iPhone à l'étranger.
-Dans l'Union Européenne, vous bénéficiez du "roaming comme à la maison", ce qui signifie que vous pouvez utiliser votre forfait français sans surcoût, dans la limite de votre contrat.
-Hors Europe, des frais de roaming et des tarifs internationaux s'appliqueront. Pour éviter des surcoûts importants, il est recommandé de désactiver les données mobiles et d'utiliser le WiFi, ou de souscrire à un pass international journalier ou hebdomadaire via votre espace client.</t>
+*   **Dans l'Union Européenne :** Vous bénéficiez du "roaming comme à la maison". Vous pouvez utiliser votre forfait français sans surcoût dans les pays de l'UE, dans les limites de votre contrat.
+*   **Hors Europe :** Des frais de roaming et des tarifs internationaux s'appliquent. Pour éviter les frais, nous vous recommandons de désactiver les données mobiles et d'utiliser le WiFi, ou de souscrire à un pass international journalier ou hebdomadaire via votre espace client.
+Le roaming international est généralement activé par défaut. Vous pouvez vérifier son statut et les tarifs applicables dans votre espace client ou en contactant notre service client.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1270,7 +1305,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>The agent's answer is accurate, complete, relevant, and very clear. It correctly distinguishes between EU and non-EU usage, explains the 'roaming comme à la maison' principle, and provides excellent practical advice for non-EU travel, including disabling mobile data/using WiFi and subscribing to an international pass via the customer area. The additional detail 'dans la limite de votre contrat' is also a good, accurate clarification. It fully addresses the user's question about using an iPhone abroad without extra cost and provides comprehensive solutions.</t>
+          <t>The agent's answer is accurate, complete, relevant, and clear. While the expected answer starts with 'Cela dépend' and the agent with 'Oui', the agent immediately qualifies the 'Oui' by differentiating between the EU (where it's 'sans surcoût') and outside Europe (where fees apply and solutions are offered). This effectively conveys the same core message. The agent also provides more helpful information (like using WiFi or checking roaming status), which is considered a positive under lenient evaluation. All key points from the expected answer are covered, and the additional details enhance the helpfulness.</t>
         </is>
       </c>
     </row>

</xml_diff>